<commit_message>
fix: modify Q1 result
</commit_message>
<xml_diff>
--- a/Q1/output/result1.xlsx
+++ b/Q1/output/result1.xlsx
@@ -1005,7 +1005,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>911.1614</v>
+        <v>577.8280</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="14" customHeight="1" ns2:dyDescent="0.25">
@@ -2085,7 +2085,7 @@
         <v>150</v>
       </c>
       <c r="B145" s="2">
-        <v>574.1210</v>
+        <v>907.4543</v>
       </c>
     </row>
   </sheetData>
@@ -2149,7 +2149,7 @@
         <v>833.3333</v>
       </c>
       <c r="C3">
-        <v>6365.8412</v>
+        <v>5947.4197</v>
       </c>
       <c r="E3">
         <v>6000.0000</v>
@@ -2160,10 +2160,10 @@
         <v>146</v>
       </c>
       <c r="B4">
-        <v>4787.9643</v>
+        <v>3954.6310</v>
       </c>
       <c r="C4">
-        <v>1702.9970</v>
+        <v>2121.4184</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="5" customFormat="1" ht="14" customHeight="1" ns2:dyDescent="0.35">
@@ -2171,7 +2171,7 @@
         <v>147</v>
       </c>
       <c r="B5">
-        <v>5286.0352</v>
+        <v>6119.3685</v>
       </c>
       <c r="C5">
         <v>91.1014</v>
@@ -2185,7 +2185,7 @@
         <v>0.0000</v>
       </c>
       <c r="C6">
-        <v>5780.1319</v>
+        <v>5068.6869</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="5" customFormat="1" ht="14" customHeight="1" ns2:dyDescent="0.35">
@@ -2196,7 +2196,7 @@
         <v>5333.3333</v>
       </c>
       <c r="C7">
-        <v>2859.8681</v>
+        <v>3571.3131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>